<commit_message>
Add 16 realistic sample transactions to the sheet
Populated the Transactions sheet with demo buy/sell records covering all
payment statuses (Paid, Pending, Due/Overdue) and delivery statuses
(Delivered, Pending) across different buyer/seller companies, products,
quantities, and dates — making the Dashboard summary live with real data.

https://claude.ai/code/session_01NbxL8TadKpbzmr71ugtmmh
</commit_message>
<xml_diff>
--- a/TransactionManagement.xlsx
+++ b/TransactionManagement.xlsx
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46101</v>
+        <v>46056</v>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
@@ -862,392 +862,1052 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="K2" s="5" t="n">
-        <v>0</v>
+        <v>25000</v>
       </c>
       <c r="L2" s="7">
         <f>IF(I2="","",I2-IF(K2="",0,K2))</f>
         <v/>
       </c>
       <c r="M2" s="3" t="n">
-        <v>46131</v>
+        <v>46086</v>
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Delivered</t>
         </is>
       </c>
       <c r="O2" s="3" t="n">
-        <v>46116</v>
+        <v>46071</v>
       </c>
       <c r="P2" s="8" t="inlineStr">
         <is>
-          <t>First order — verify quality before full payment</t>
+          <t>Bulk order for new office wing</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="n"/>
-      <c r="B3" s="10" t="n"/>
-      <c r="C3" s="11" t="n"/>
-      <c r="D3" s="11" t="n"/>
-      <c r="E3" s="11" t="n"/>
-      <c r="F3" s="11" t="n"/>
-      <c r="G3" s="9" t="n"/>
-      <c r="H3" s="12" t="n"/>
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>TXN-0002</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="n">
+        <v>46071</v>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Sunrise Retail Co.</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>LED Strip Lights</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="H3" s="12" t="n">
+        <v>350</v>
+      </c>
       <c r="I3" s="13">
         <f>IF(G3*H3=0,"",G3*H3)</f>
         <v/>
       </c>
-      <c r="J3" s="11" t="n"/>
-      <c r="K3" s="12" t="n"/>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="K3" s="12" t="n">
+        <v>17500</v>
+      </c>
       <c r="L3" s="14">
         <f>IF(I3="","",I3-IF(K3="",0,K3))</f>
         <v/>
       </c>
-      <c r="M3" s="10" t="n"/>
-      <c r="N3" s="11" t="n"/>
-      <c r="O3" s="10" t="n"/>
-      <c r="P3" s="15" t="n"/>
+      <c r="M3" s="10" t="n">
+        <v>46091</v>
+      </c>
+      <c r="N3" s="11" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="O3" s="10" t="n">
+        <v>46081</v>
+      </c>
+      <c r="P3" s="15" t="inlineStr">
+        <is>
+          <t>Monthly supply contract</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="5" t="n"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>TXN-0003</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>46081</v>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Metro Supplies Ltd.</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>A4 Paper (Box)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>480</v>
+      </c>
       <c r="I4" s="6">
         <f>IF(G4*H4=0,"",G4*H4)</f>
         <v/>
       </c>
-      <c r="J4" s="4" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>48000</v>
+      </c>
       <c r="L4" s="7">
         <f>IF(I4="","",I4-IF(K4="",0,K4))</f>
         <v/>
       </c>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="4" t="n"/>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="8" t="n"/>
+      <c r="M4" s="3" t="n">
+        <v>46096</v>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>46089</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Stationery restock Q1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n"/>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="11" t="n"/>
-      <c r="D5" s="11" t="n"/>
-      <c r="E5" s="11" t="n"/>
-      <c r="F5" s="11" t="n"/>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="12" t="n"/>
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>TXN-0004</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>46083</v>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Greenleaf Corp.</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Laptop Bags</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="H5" s="12" t="n">
+        <v>750</v>
+      </c>
       <c r="I5" s="13">
         <f>IF(G5*H5=0,"",G5*H5)</f>
         <v/>
       </c>
-      <c r="J5" s="11" t="n"/>
-      <c r="K5" s="12" t="n"/>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>22500</v>
+      </c>
       <c r="L5" s="14">
         <f>IF(I5="","",I5-IF(K5="",0,K5))</f>
         <v/>
       </c>
-      <c r="M5" s="10" t="n"/>
-      <c r="N5" s="11" t="n"/>
-      <c r="O5" s="10" t="n"/>
-      <c r="P5" s="15" t="n"/>
+      <c r="M5" s="10" t="n">
+        <v>46093</v>
+      </c>
+      <c r="N5" s="11" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="O5" s="10" t="n">
+        <v>46086</v>
+      </c>
+      <c r="P5" s="15" t="inlineStr">
+        <is>
+          <t>Corporate gift order</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TXN-0005</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>46086</v>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>TechZone Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>USB-C Hubs</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>1200</v>
+      </c>
       <c r="I6" s="6">
         <f>IF(G6*H6=0,"",G6*H6)</f>
         <v/>
       </c>
-      <c r="J6" s="4" t="n"/>
-      <c r="K6" s="5" t="n"/>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L6" s="7">
         <f>IF(I6="","",I6-IF(K6="",0,K6))</f>
         <v/>
       </c>
-      <c r="M6" s="3" t="n"/>
-      <c r="N6" s="4" t="n"/>
-      <c r="O6" s="3" t="n"/>
-      <c r="P6" s="8" t="n"/>
+      <c r="M6" s="3" t="n">
+        <v>46116</v>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>46111</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Awaiting delivery confirmation</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n"/>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="11" t="n"/>
-      <c r="E7" s="11" t="n"/>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="12" t="n"/>
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>TXN-0006</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>46089</v>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>BlueStar Industries</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Printer Cartridges</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="H7" s="12" t="n">
+        <v>320</v>
+      </c>
       <c r="I7" s="13">
         <f>IF(G7*H7=0,"",G7*H7)</f>
         <v/>
       </c>
-      <c r="J7" s="11" t="n"/>
-      <c r="K7" s="12" t="n"/>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="n">
+        <v>0</v>
+      </c>
       <c r="L7" s="14">
         <f>IF(I7="","",I7-IF(K7="",0,K7))</f>
         <v/>
       </c>
-      <c r="M7" s="10" t="n"/>
-      <c r="N7" s="11" t="n"/>
-      <c r="O7" s="10" t="n"/>
-      <c r="P7" s="15" t="n"/>
+      <c r="M7" s="10" t="n">
+        <v>46119</v>
+      </c>
+      <c r="N7" s="11" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="O7" s="10" t="n">
+        <v>46096</v>
+      </c>
+      <c r="P7" s="15" t="inlineStr">
+        <is>
+          <t>Invoice sent; awaiting payment</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="3" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="5" t="n"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>TXN-0007</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>46091</v>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Global Furniture Co.</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Standing Desks</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>8500</v>
+      </c>
       <c r="I8" s="6">
         <f>IF(G8*H8=0,"",G8*H8)</f>
         <v/>
       </c>
-      <c r="J8" s="4" t="n"/>
-      <c r="K8" s="5" t="n"/>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>34000</v>
+      </c>
       <c r="L8" s="7">
         <f>IF(I8="","",I8-IF(K8="",0,K8))</f>
         <v/>
       </c>
-      <c r="M8" s="3" t="n"/>
-      <c r="N8" s="4" t="n"/>
-      <c r="O8" s="3" t="n"/>
-      <c r="P8" s="8" t="n"/>
+      <c r="M8" s="3" t="n">
+        <v>46121</v>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>46126</v>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>Partial advance paid; balance on delivery</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n"/>
-      <c r="B9" s="10" t="n"/>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="9" t="n"/>
-      <c r="H9" s="12" t="n"/>
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>TXN-0008</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>46093</v>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Horizon Traders</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>Wireless Keyboards</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="n">
+        <v>25</v>
+      </c>
+      <c r="H9" s="12" t="n">
+        <v>950</v>
+      </c>
       <c r="I9" s="13">
         <f>IF(G9*H9=0,"",G9*H9)</f>
         <v/>
       </c>
-      <c r="J9" s="11" t="n"/>
-      <c r="K9" s="12" t="n"/>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>0</v>
+      </c>
       <c r="L9" s="14">
         <f>IF(I9="","",I9-IF(K9="",0,K9))</f>
         <v/>
       </c>
-      <c r="M9" s="10" t="n"/>
-      <c r="N9" s="11" t="n"/>
-      <c r="O9" s="10" t="n"/>
-      <c r="P9" s="15" t="n"/>
+      <c r="M9" s="10" t="n">
+        <v>46113</v>
+      </c>
+      <c r="N9" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O9" s="10" t="n">
+        <v>46109</v>
+      </c>
+      <c r="P9" s="15" t="inlineStr">
+        <is>
+          <t>Order confirmed; production in progress</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="3" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>TXN-0009</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>46066</v>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Speedy Logistics</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Packaging Material</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>200</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>150</v>
+      </c>
       <c r="I10" s="6">
         <f>IF(G10*H10=0,"",G10*H10)</f>
         <v/>
       </c>
-      <c r="J10" s="4" t="n"/>
-      <c r="K10" s="5" t="n"/>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>Due</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L10" s="7">
         <f>IF(I10="","",I10-IF(K10="",0,K10))</f>
         <v/>
       </c>
-      <c r="M10" s="3" t="n"/>
-      <c r="N10" s="4" t="n"/>
-      <c r="O10" s="3" t="n"/>
-      <c r="P10" s="8" t="n"/>
+      <c r="M10" s="3" t="n">
+        <v>46091</v>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>46073</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>Payment overdue — follow up with accounts</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="10" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="9" t="n"/>
-      <c r="H11" s="12" t="n"/>
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>TXN-0010</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>46076</v>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Redwood Distributors</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Steel Shelving Units</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="H11" s="12" t="n">
+        <v>3200</v>
+      </c>
       <c r="I11" s="13">
         <f>IF(G11*H11=0,"",G11*H11)</f>
         <v/>
       </c>
-      <c r="J11" s="11" t="n"/>
-      <c r="K11" s="12" t="n"/>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>Due</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>16000</v>
+      </c>
       <c r="L11" s="14">
         <f>IF(I11="","",I11-IF(K11="",0,K11))</f>
         <v/>
       </c>
-      <c r="M11" s="10" t="n"/>
-      <c r="N11" s="11" t="n"/>
-      <c r="O11" s="10" t="n"/>
-      <c r="P11" s="15" t="n"/>
+      <c r="M11" s="10" t="n">
+        <v>46096</v>
+      </c>
+      <c r="N11" s="11" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="O11" s="10" t="n">
+        <v>46083</v>
+      </c>
+      <c r="P11" s="15" t="inlineStr">
+        <is>
+          <t>Partial payment received; balance due</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="5" t="n"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TXN-0011</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>46079</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Alpha Electronics</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>HDMI Cables (pack)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>220</v>
+      </c>
       <c r="I12" s="6">
         <f>IF(G12*H12=0,"",G12*H12)</f>
         <v/>
       </c>
-      <c r="J12" s="4" t="n"/>
-      <c r="K12" s="5" t="n"/>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Due</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>0</v>
+      </c>
       <c r="L12" s="7">
         <f>IF(I12="","",I12-IF(K12="",0,K12))</f>
         <v/>
       </c>
-      <c r="M12" s="3" t="n"/>
-      <c r="N12" s="4" t="n"/>
-      <c r="O12" s="3" t="n"/>
-      <c r="P12" s="8" t="n"/>
+      <c r="M12" s="3" t="n">
+        <v>46099</v>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>46081</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>Urgent: payment deadline crossed</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="9" t="n"/>
-      <c r="H13" s="12" t="n"/>
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>TXN-0012</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>46096</v>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Pinnacle Group</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>Office Sofas</t>
+        </is>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H13" s="12" t="n">
+        <v>12000</v>
+      </c>
       <c r="I13" s="13">
         <f>IF(G13*H13=0,"",G13*H13)</f>
         <v/>
       </c>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="12" t="n"/>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K13" s="12" t="n">
+        <v>0</v>
+      </c>
       <c r="L13" s="14">
         <f>IF(I13="","",I13-IF(K13="",0,K13))</f>
         <v/>
       </c>
-      <c r="M13" s="10" t="n"/>
-      <c r="N13" s="11" t="n"/>
-      <c r="O13" s="10" t="n"/>
-      <c r="P13" s="15" t="n"/>
+      <c r="M13" s="10" t="n">
+        <v>46131</v>
+      </c>
+      <c r="N13" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O13" s="10" t="n">
+        <v>46146</v>
+      </c>
+      <c r="P13" s="15" t="inlineStr">
+        <is>
+          <t>Custom order; 45-day delivery window</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="5" t="n"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TXN-0013</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>46098</v>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>SwiftPrint Solutions</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Business Cards (500)</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>800</v>
+      </c>
       <c r="I14" s="6">
         <f>IF(G14*H14=0,"",G14*H14)</f>
         <v/>
       </c>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="5" t="n"/>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>3200</v>
+      </c>
       <c r="L14" s="7">
         <f>IF(I14="","",I14-IF(K14="",0,K14))</f>
         <v/>
       </c>
-      <c r="M14" s="3" t="n"/>
-      <c r="N14" s="4" t="n"/>
-      <c r="O14" s="3" t="n"/>
-      <c r="P14" s="8" t="n"/>
+      <c r="M14" s="3" t="n">
+        <v>46101</v>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>46106</v>
+      </c>
+      <c r="P14" s="8" t="inlineStr">
+        <is>
+          <t>Branding refresh batch</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="n"/>
-      <c r="B15" s="10" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="9" t="n"/>
-      <c r="H15" s="12" t="n"/>
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>TXN-0014</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>46099</v>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Nexus Retail Ltd.</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Extension Cords</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="n">
+        <v>100</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>180</v>
+      </c>
       <c r="I15" s="13">
         <f>IF(G15*H15=0,"",G15*H15)</f>
         <v/>
       </c>
-      <c r="J15" s="11" t="n"/>
-      <c r="K15" s="12" t="n"/>
+      <c r="J15" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>0</v>
+      </c>
       <c r="L15" s="14">
         <f>IF(I15="","",I15-IF(K15="",0,K15))</f>
         <v/>
       </c>
-      <c r="M15" s="10" t="n"/>
-      <c r="N15" s="11" t="n"/>
-      <c r="O15" s="10" t="n"/>
-      <c r="P15" s="15" t="n"/>
+      <c r="M15" s="10" t="n">
+        <v>46122</v>
+      </c>
+      <c r="N15" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O15" s="10" t="n">
+        <v>46115</v>
+      </c>
+      <c r="P15" s="15" t="inlineStr">
+        <is>
+          <t>New client — net-30 payment terms</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="5" t="n"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TXN-0015</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>46100</v>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Buy</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>CloudServe India</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Annual SaaS License</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>85000</v>
+      </c>
       <c r="I16" s="6">
         <f>IF(G16*H16=0,"",G16*H16)</f>
         <v/>
       </c>
-      <c r="J16" s="4" t="n"/>
-      <c r="K16" s="5" t="n"/>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="n">
+        <v>85000</v>
+      </c>
       <c r="L16" s="7">
         <f>IF(I16="","",I16-IF(K16="",0,K16))</f>
         <v/>
       </c>
-      <c r="M16" s="3" t="n"/>
-      <c r="N16" s="4" t="n"/>
-      <c r="O16" s="3" t="n"/>
-      <c r="P16" s="8" t="n"/>
+      <c r="M16" s="3" t="n">
+        <v>46101</v>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>Delivered</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>46100</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>Annual ERP renewal — auto-renews next year</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="9" t="n"/>
-      <c r="B17" s="10" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="9" t="n"/>
-      <c r="H17" s="12" t="n"/>
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>TXN-0016</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>46101</v>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Sell</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Eastgate Wholesalers</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>ABC Enterprises</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Projector Screens</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="H17" s="12" t="n">
+        <v>4500</v>
+      </c>
       <c r="I17" s="13">
         <f>IF(G17*H17=0,"",G17*H17)</f>
         <v/>
       </c>
-      <c r="J17" s="11" t="n"/>
-      <c r="K17" s="12" t="n"/>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>0</v>
+      </c>
       <c r="L17" s="14">
         <f>IF(I17="","",I17-IF(K17="",0,K17))</f>
         <v/>
       </c>
-      <c r="M17" s="10" t="n"/>
-      <c r="N17" s="11" t="n"/>
-      <c r="O17" s="10" t="n"/>
-      <c r="P17" s="15" t="n"/>
+      <c r="M17" s="10" t="n">
+        <v>46116</v>
+      </c>
+      <c r="N17" s="11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="O17" s="10" t="n">
+        <v>46121</v>
+      </c>
+      <c r="P17" s="15" t="inlineStr">
+        <is>
+          <t>New bulk deal — first transaction</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n"/>

</xml_diff>